<commit_message>
02 Completed Revenue & Quantity Analysis
</commit_message>
<xml_diff>
--- a/sales-dataset.xlsx
+++ b/sales-dataset.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\franc\OneDrive\Desktop\DATA SCIENCE\20 Beginner Excel Data Analyst Practice Questions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\franc\OneDrive\Desktop\DATA SCIENCE\20 Beginner Excel Data Analyst Practice Questions\20_beginner_excel_data_analyst_practice_questions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{375AC8DB-D1F0-416A-BC39-73DA4215B3F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D511DF7-98F1-424B-B695-73FE49B6842B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,8 +18,19 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Raw_Sales_Data!$A$1:$J$51</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -28,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="96">
   <si>
     <t>Order_ID</t>
   </si>
@@ -307,6 +318,15 @@
   </si>
   <si>
     <t>Imran Khan</t>
+  </si>
+  <si>
+    <t>Revenue</t>
+  </si>
+  <si>
+    <t>Total_Sales</t>
+  </si>
+  <si>
+    <t>Total_Quantity_Sold</t>
   </si>
 </sst>
 </file>
@@ -314,9 +334,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -329,6 +349,14 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -338,7 +366,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -361,16 +389,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -673,7 +716,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -686,9 +729,10 @@
     <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="16" customWidth="1"/>
     <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="12" max="12" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -719,8 +763,14 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1001</v>
       </c>
@@ -751,8 +801,16 @@
       <c r="J2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K2">
+        <f>H2*G2</f>
+        <v>170000</v>
+      </c>
+      <c r="L2">
+        <f>SUM(K2:K51)</f>
+        <v>5189800</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1002</v>
       </c>
@@ -783,8 +841,12 @@
       <c r="J3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K3">
+        <f t="shared" ref="K3:K51" si="0">H3*G3</f>
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1003</v>
       </c>
@@ -815,8 +877,15 @@
       <c r="J4" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K4">
+        <f t="shared" si="0"/>
+        <v>25000</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1004</v>
       </c>
@@ -847,8 +916,16 @@
       <c r="J5" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K5">
+        <f t="shared" si="0"/>
+        <v>25500</v>
+      </c>
+      <c r="L5">
+        <f>SUM(G2:G51)</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1005</v>
       </c>
@@ -879,8 +956,12 @@
       <c r="J6" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K6">
+        <f t="shared" si="0"/>
+        <v>64000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1006</v>
       </c>
@@ -911,8 +992,12 @@
       <c r="J7" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K7">
+        <f t="shared" si="0"/>
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1007</v>
       </c>
@@ -943,8 +1028,12 @@
       <c r="J8" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K8">
+        <f t="shared" si="0"/>
+        <v>26000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1008</v>
       </c>
@@ -975,8 +1064,12 @@
       <c r="J9" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K9">
+        <f t="shared" si="0"/>
+        <v>27000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>1009</v>
       </c>
@@ -1007,8 +1100,12 @@
       <c r="J10" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K10">
+        <f t="shared" si="0"/>
+        <v>56000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1010</v>
       </c>
@@ -1039,8 +1136,12 @@
       <c r="J11" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K11">
+        <f t="shared" si="0"/>
+        <v>27500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>1011</v>
       </c>
@@ -1071,8 +1172,12 @@
       <c r="J12" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K12">
+        <f t="shared" si="0"/>
+        <v>96000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1012</v>
       </c>
@@ -1103,8 +1208,12 @@
       <c r="J13" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K13">
+        <f t="shared" si="0"/>
+        <v>95000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>1013</v>
       </c>
@@ -1135,8 +1244,12 @@
       <c r="J14" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K14">
+        <f t="shared" si="0"/>
+        <v>92000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1014</v>
       </c>
@@ -1167,8 +1280,12 @@
       <c r="J15" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K15">
+        <f t="shared" si="0"/>
+        <v>33600</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>1015</v>
       </c>
@@ -1199,8 +1316,12 @@
       <c r="J16" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K16">
+        <f t="shared" si="0"/>
+        <v>165000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>1016</v>
       </c>
@@ -1231,8 +1352,12 @@
       <c r="J17" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K17">
+        <f t="shared" si="0"/>
+        <v>125000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>1017</v>
       </c>
@@ -1263,8 +1388,12 @@
       <c r="J18" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K18">
+        <f t="shared" si="0"/>
+        <v>38400</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>1018</v>
       </c>
@@ -1295,8 +1424,12 @@
       <c r="J19" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K19">
+        <f t="shared" si="0"/>
+        <v>52500</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>1019</v>
       </c>
@@ -1327,8 +1460,12 @@
       <c r="J20" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K20">
+        <f t="shared" si="0"/>
+        <v>54000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>1020</v>
       </c>
@@ -1359,8 +1496,12 @@
       <c r="J21" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K21">
+        <f t="shared" si="0"/>
+        <v>36000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>1021</v>
       </c>
@@ -1391,8 +1532,12 @@
       <c r="J22" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K22">
+        <f t="shared" si="0"/>
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>1022</v>
       </c>
@@ -1423,8 +1568,12 @@
       <c r="J23" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K23">
+        <f t="shared" si="0"/>
+        <v>115000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>1023</v>
       </c>
@@ -1455,8 +1604,12 @@
       <c r="J24" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K24">
+        <f t="shared" si="0"/>
+        <v>176000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>1024</v>
       </c>
@@ -1487,8 +1640,12 @@
       <c r="J25" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K25">
+        <f t="shared" si="0"/>
+        <v>46800</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>1025</v>
       </c>
@@ -1519,8 +1676,12 @@
       <c r="J26" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K26">
+        <f t="shared" si="0"/>
+        <v>136000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>1026</v>
       </c>
@@ -1551,8 +1712,12 @@
       <c r="J27" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K27">
+        <f t="shared" si="0"/>
+        <v>63000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>1027</v>
       </c>
@@ -1583,8 +1748,12 @@
       <c r="J28" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K28">
+        <f t="shared" si="0"/>
+        <v>49200</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>1028</v>
       </c>
@@ -1615,8 +1784,12 @@
       <c r="J29" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K29">
+        <f t="shared" si="0"/>
+        <v>126000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>1029</v>
       </c>
@@ -1647,8 +1820,12 @@
       <c r="J30" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K30">
+        <f t="shared" si="0"/>
+        <v>208000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>1030</v>
       </c>
@@ -1679,8 +1856,12 @@
       <c r="J31" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K31">
+        <f t="shared" si="0"/>
+        <v>54400</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>1031</v>
       </c>
@@ -1711,8 +1892,12 @@
       <c r="J32" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K32">
+        <f t="shared" si="0"/>
+        <v>230000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>1032</v>
       </c>
@@ -1743,8 +1928,12 @@
       <c r="J33" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K33">
+        <f t="shared" si="0"/>
+        <v>135000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>1033</v>
       </c>
@@ -1775,8 +1964,12 @@
       <c r="J34" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K34">
+        <f t="shared" si="0"/>
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>1034</v>
       </c>
@@ -1807,8 +2000,12 @@
       <c r="J35" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K35">
+        <f t="shared" si="0"/>
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>1035</v>
       </c>
@@ -1839,8 +2036,12 @@
       <c r="J36" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K36">
+        <f t="shared" si="0"/>
+        <v>184000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>1036</v>
       </c>
@@ -1871,8 +2072,12 @@
       <c r="J37" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K37">
+        <f t="shared" si="0"/>
+        <v>86400</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>1037</v>
       </c>
@@ -1903,8 +2108,12 @@
       <c r="J38" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K38">
+        <f t="shared" si="0"/>
+        <v>61600</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>1038</v>
       </c>
@@ -1935,8 +2144,12 @@
       <c r="J39" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K39">
+        <f t="shared" si="0"/>
+        <v>108000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>1039</v>
       </c>
@@ -1967,8 +2180,12 @@
       <c r="J40" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K40">
+        <f t="shared" si="0"/>
+        <v>270000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>1040</v>
       </c>
@@ -1999,8 +2216,12 @@
       <c r="J41" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K41">
+        <f t="shared" si="0"/>
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>1041</v>
       </c>
@@ -2031,8 +2252,12 @@
       <c r="J42" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K42">
+        <f t="shared" si="0"/>
+        <v>177000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>1042</v>
       </c>
@@ -2063,8 +2288,12 @@
       <c r="J43" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K43">
+        <f t="shared" si="0"/>
+        <v>126000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>1043</v>
       </c>
@@ -2095,8 +2324,12 @@
       <c r="J44" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K44">
+        <f t="shared" si="0"/>
+        <v>58300</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>1044</v>
       </c>
@@ -2127,8 +2360,12 @@
       <c r="J45" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K45">
+        <f t="shared" si="0"/>
+        <v>195000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>1045</v>
       </c>
@@ -2159,8 +2396,12 @@
       <c r="J46" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K46">
+        <f t="shared" si="0"/>
+        <v>324000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>1046</v>
       </c>
@@ -2191,8 +2432,12 @@
       <c r="J47" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K47">
+        <f t="shared" si="0"/>
+        <v>43000</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>1047</v>
       </c>
@@ -2223,8 +2468,12 @@
       <c r="J48" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K48">
+        <f t="shared" si="0"/>
+        <v>172000</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>1048</v>
       </c>
@@ -2255,8 +2504,12 @@
       <c r="J49" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K49">
+        <f t="shared" si="0"/>
+        <v>141000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>1049</v>
       </c>
@@ -2287,8 +2540,12 @@
       <c r="J50" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K50">
+        <f t="shared" si="0"/>
+        <v>89600</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>1050</v>
       </c>
@@ -2318,6 +2575,10 @@
       </c>
       <c r="J51" t="s">
         <v>29</v>
+      </c>
+      <c r="K51">
+        <f t="shared" si="0"/>
+        <v>256000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
03 Completed Level 1 Excel Analysis
</commit_message>
<xml_diff>
--- a/sales-dataset.xlsx
+++ b/sales-dataset.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\franc\OneDrive\Desktop\DATA SCIENCE\20 Beginner Excel Data Analyst Practice Questions\20_beginner_excel_data_analyst_practice_questions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D511DF7-98F1-424B-B695-73FE49B6842B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B870353A-4F69-4440-A95A-24B5EC5931CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Sales_Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Analysis" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Raw_Sales_Data!$A$1:$J$51</definedName>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="98">
   <si>
     <t>Order_ID</t>
   </si>
@@ -327,6 +328,12 @@
   </si>
   <si>
     <t>Total_Quantity_Sold</t>
+  </si>
+  <si>
+    <t>Average_Order_Revenue</t>
+  </si>
+  <si>
+    <t>Highest_Order_Value</t>
   </si>
 </sst>
 </file>
@@ -716,7 +723,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -729,10 +736,9 @@
     <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="16" customWidth="1"/>
     <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="12" max="12" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -763,14 +769,8 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1001</v>
       </c>
@@ -801,16 +801,8 @@
       <c r="J2" t="s">
         <v>15</v>
       </c>
-      <c r="K2">
-        <f>H2*G2</f>
-        <v>170000</v>
-      </c>
-      <c r="L2">
-        <f>SUM(K2:K51)</f>
-        <v>5189800</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1002</v>
       </c>
@@ -841,12 +833,8 @@
       <c r="J3" t="s">
         <v>21</v>
       </c>
-      <c r="K3">
-        <f t="shared" ref="K3:K51" si="0">H3*G3</f>
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1003</v>
       </c>
@@ -877,15 +865,8 @@
       <c r="J4" t="s">
         <v>15</v>
       </c>
-      <c r="K4">
-        <f t="shared" si="0"/>
-        <v>25000</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1004</v>
       </c>
@@ -916,16 +897,8 @@
       <c r="J5" t="s">
         <v>29</v>
       </c>
-      <c r="K5">
-        <f t="shared" si="0"/>
-        <v>25500</v>
-      </c>
-      <c r="L5">
-        <f>SUM(G2:G51)</f>
-        <v>300</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1005</v>
       </c>
@@ -956,12 +929,8 @@
       <c r="J6" t="s">
         <v>15</v>
       </c>
-      <c r="K6">
-        <f t="shared" si="0"/>
-        <v>64000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1006</v>
       </c>
@@ -992,12 +961,8 @@
       <c r="J7" t="s">
         <v>21</v>
       </c>
-      <c r="K7">
-        <f t="shared" si="0"/>
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1007</v>
       </c>
@@ -1028,12 +993,8 @@
       <c r="J8" t="s">
         <v>15</v>
       </c>
-      <c r="K8">
-        <f t="shared" si="0"/>
-        <v>26000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1008</v>
       </c>
@@ -1064,12 +1025,8 @@
       <c r="J9" t="s">
         <v>29</v>
       </c>
-      <c r="K9">
-        <f t="shared" si="0"/>
-        <v>27000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>1009</v>
       </c>
@@ -1100,12 +1057,8 @@
       <c r="J10" t="s">
         <v>21</v>
       </c>
-      <c r="K10">
-        <f t="shared" si="0"/>
-        <v>56000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1010</v>
       </c>
@@ -1136,12 +1089,8 @@
       <c r="J11" t="s">
         <v>15</v>
       </c>
-      <c r="K11">
-        <f t="shared" si="0"/>
-        <v>27500</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>1011</v>
       </c>
@@ -1172,12 +1121,8 @@
       <c r="J12" t="s">
         <v>15</v>
       </c>
-      <c r="K12">
-        <f t="shared" si="0"/>
-        <v>96000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1012</v>
       </c>
@@ -1208,12 +1153,8 @@
       <c r="J13" t="s">
         <v>29</v>
       </c>
-      <c r="K13">
-        <f t="shared" si="0"/>
-        <v>95000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>1013</v>
       </c>
@@ -1244,12 +1185,8 @@
       <c r="J14" t="s">
         <v>15</v>
       </c>
-      <c r="K14">
-        <f t="shared" si="0"/>
-        <v>92000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1014</v>
       </c>
@@ -1280,12 +1217,8 @@
       <c r="J15" t="s">
         <v>21</v>
       </c>
-      <c r="K15">
-        <f t="shared" si="0"/>
-        <v>33600</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>1015</v>
       </c>
@@ -1316,12 +1249,8 @@
       <c r="J16" t="s">
         <v>15</v>
       </c>
-      <c r="K16">
-        <f t="shared" si="0"/>
-        <v>165000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>1016</v>
       </c>
@@ -1352,12 +1281,8 @@
       <c r="J17" t="s">
         <v>29</v>
       </c>
-      <c r="K17">
-        <f t="shared" si="0"/>
-        <v>125000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>1017</v>
       </c>
@@ -1388,12 +1313,8 @@
       <c r="J18" t="s">
         <v>21</v>
       </c>
-      <c r="K18">
-        <f t="shared" si="0"/>
-        <v>38400</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>1018</v>
       </c>
@@ -1424,12 +1345,8 @@
       <c r="J19" t="s">
         <v>15</v>
       </c>
-      <c r="K19">
-        <f t="shared" si="0"/>
-        <v>52500</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>1019</v>
       </c>
@@ -1460,12 +1377,8 @@
       <c r="J20" t="s">
         <v>21</v>
       </c>
-      <c r="K20">
-        <f t="shared" si="0"/>
-        <v>54000</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>1020</v>
       </c>
@@ -1496,12 +1409,8 @@
       <c r="J21" t="s">
         <v>29</v>
       </c>
-      <c r="K21">
-        <f t="shared" si="0"/>
-        <v>36000</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>1021</v>
       </c>
@@ -1532,12 +1441,8 @@
       <c r="J22" t="s">
         <v>15</v>
       </c>
-      <c r="K22">
-        <f t="shared" si="0"/>
-        <v>90000</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>1022</v>
       </c>
@@ -1568,12 +1473,8 @@
       <c r="J23" t="s">
         <v>21</v>
       </c>
-      <c r="K23">
-        <f t="shared" si="0"/>
-        <v>115000</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>1023</v>
       </c>
@@ -1604,12 +1505,8 @@
       <c r="J24" t="s">
         <v>29</v>
       </c>
-      <c r="K24">
-        <f t="shared" si="0"/>
-        <v>176000</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>1024</v>
       </c>
@@ -1640,12 +1537,8 @@
       <c r="J25" t="s">
         <v>15</v>
       </c>
-      <c r="K25">
-        <f t="shared" si="0"/>
-        <v>46800</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>1025</v>
       </c>
@@ -1676,12 +1569,8 @@
       <c r="J26" t="s">
         <v>15</v>
       </c>
-      <c r="K26">
-        <f t="shared" si="0"/>
-        <v>136000</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>1026</v>
       </c>
@@ -1712,12 +1601,8 @@
       <c r="J27" t="s">
         <v>21</v>
       </c>
-      <c r="K27">
-        <f t="shared" si="0"/>
-        <v>63000</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>1027</v>
       </c>
@@ -1748,12 +1633,8 @@
       <c r="J28" t="s">
         <v>15</v>
       </c>
-      <c r="K28">
-        <f t="shared" si="0"/>
-        <v>49200</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>1028</v>
       </c>
@@ -1784,12 +1665,8 @@
       <c r="J29" t="s">
         <v>29</v>
       </c>
-      <c r="K29">
-        <f t="shared" si="0"/>
-        <v>126000</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>1029</v>
       </c>
@@ -1820,12 +1697,8 @@
       <c r="J30" t="s">
         <v>15</v>
       </c>
-      <c r="K30">
-        <f t="shared" si="0"/>
-        <v>208000</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>1030</v>
       </c>
@@ -1856,12 +1729,8 @@
       <c r="J31" t="s">
         <v>21</v>
       </c>
-      <c r="K31">
-        <f t="shared" si="0"/>
-        <v>54400</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>1031</v>
       </c>
@@ -1892,12 +1761,8 @@
       <c r="J32" t="s">
         <v>15</v>
       </c>
-      <c r="K32">
-        <f t="shared" si="0"/>
-        <v>230000</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>1032</v>
       </c>
@@ -1928,12 +1793,8 @@
       <c r="J33" t="s">
         <v>29</v>
       </c>
-      <c r="K33">
-        <f t="shared" si="0"/>
-        <v>135000</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>1033</v>
       </c>
@@ -1964,12 +1825,8 @@
       <c r="J34" t="s">
         <v>21</v>
       </c>
-      <c r="K34">
-        <f t="shared" si="0"/>
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>1034</v>
       </c>
@@ -2000,12 +1857,8 @@
       <c r="J35" t="s">
         <v>15</v>
       </c>
-      <c r="K35">
-        <f t="shared" si="0"/>
-        <v>55000</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>1035</v>
       </c>
@@ -2036,12 +1889,8 @@
       <c r="J36" t="s">
         <v>29</v>
       </c>
-      <c r="K36">
-        <f t="shared" si="0"/>
-        <v>184000</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>1036</v>
       </c>
@@ -2072,12 +1921,8 @@
       <c r="J37" t="s">
         <v>15</v>
       </c>
-      <c r="K37">
-        <f t="shared" si="0"/>
-        <v>86400</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>1037</v>
       </c>
@@ -2108,12 +1953,8 @@
       <c r="J38" t="s">
         <v>21</v>
       </c>
-      <c r="K38">
-        <f t="shared" si="0"/>
-        <v>61600</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>1038</v>
       </c>
@@ -2144,12 +1985,8 @@
       <c r="J39" t="s">
         <v>15</v>
       </c>
-      <c r="K39">
-        <f t="shared" si="0"/>
-        <v>108000</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>1039</v>
       </c>
@@ -2180,12 +2017,8 @@
       <c r="J40" t="s">
         <v>29</v>
       </c>
-      <c r="K40">
-        <f t="shared" si="0"/>
-        <v>270000</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>1040</v>
       </c>
@@ -2216,12 +2049,8 @@
       <c r="J41" t="s">
         <v>21</v>
       </c>
-      <c r="K41">
-        <f t="shared" si="0"/>
-        <v>40000</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>1041</v>
       </c>
@@ -2252,12 +2081,8 @@
       <c r="J42" t="s">
         <v>15</v>
       </c>
-      <c r="K42">
-        <f t="shared" si="0"/>
-        <v>177000</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>1042</v>
       </c>
@@ -2288,12 +2113,8 @@
       <c r="J43" t="s">
         <v>15</v>
       </c>
-      <c r="K43">
-        <f t="shared" si="0"/>
-        <v>126000</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>1043</v>
       </c>
@@ -2324,12 +2145,8 @@
       <c r="J44" t="s">
         <v>29</v>
       </c>
-      <c r="K44">
-        <f t="shared" si="0"/>
-        <v>58300</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>1044</v>
       </c>
@@ -2360,12 +2177,8 @@
       <c r="J45" t="s">
         <v>21</v>
       </c>
-      <c r="K45">
-        <f t="shared" si="0"/>
-        <v>195000</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>1045</v>
       </c>
@@ -2396,12 +2209,8 @@
       <c r="J46" t="s">
         <v>15</v>
       </c>
-      <c r="K46">
-        <f t="shared" si="0"/>
-        <v>324000</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>1046</v>
       </c>
@@ -2432,12 +2241,8 @@
       <c r="J47" t="s">
         <v>21</v>
       </c>
-      <c r="K47">
-        <f t="shared" si="0"/>
-        <v>43000</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>1047</v>
       </c>
@@ -2468,12 +2273,8 @@
       <c r="J48" t="s">
         <v>29</v>
       </c>
-      <c r="K48">
-        <f t="shared" si="0"/>
-        <v>172000</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>1048</v>
       </c>
@@ -2504,12 +2305,8 @@
       <c r="J49" t="s">
         <v>15</v>
       </c>
-      <c r="K49">
-        <f t="shared" si="0"/>
-        <v>141000</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>1049</v>
       </c>
@@ -2540,12 +2337,8 @@
       <c r="J50" t="s">
         <v>21</v>
       </c>
-      <c r="K50">
-        <f t="shared" si="0"/>
-        <v>89600</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>1050</v>
       </c>
@@ -2575,14 +2368,358 @@
       </c>
       <c r="J51" t="s">
         <v>29</v>
-      </c>
-      <c r="K51">
-        <f t="shared" si="0"/>
-        <v>256000</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J51" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{754E7F86-FEF9-4E04-B3AF-20B05D640C6F}">
+  <dimension ref="A1:B51"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="2" max="2" width="22.33203125" customWidth="1"/>
+    <col min="3" max="3" width="20.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <f>Raw_Sales_Data!H2*Raw_Sales_Data!G2</f>
+        <v>170000</v>
+      </c>
+      <c r="B2">
+        <f>SUM(Analysis!A2:A51)</f>
+        <v>5189800</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <f>Raw_Sales_Data!H3*Raw_Sales_Data!G3</f>
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <f>Raw_Sales_Data!H4*Raw_Sales_Data!G4</f>
+        <v>25000</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <f>Raw_Sales_Data!H5*Raw_Sales_Data!G5</f>
+        <v>25500</v>
+      </c>
+      <c r="B5">
+        <f>SUM(Raw_Sales_Data!G2:G51)</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <f>Raw_Sales_Data!H6*Raw_Sales_Data!G6</f>
+        <v>64000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <f>Raw_Sales_Data!H7*Raw_Sales_Data!G7</f>
+        <v>45000</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <f>Raw_Sales_Data!H8*Raw_Sales_Data!G8</f>
+        <v>26000</v>
+      </c>
+      <c r="B8">
+        <f>AVERAGE(Analysis!A:A)</f>
+        <v>103796</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <f>Raw_Sales_Data!H9*Raw_Sales_Data!G9</f>
+        <v>27000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <f>Raw_Sales_Data!H10*Raw_Sales_Data!G10</f>
+        <v>56000</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <f>Raw_Sales_Data!H11*Raw_Sales_Data!G11</f>
+        <v>27500</v>
+      </c>
+      <c r="B11">
+        <f>MAX(Analysis!A:A)</f>
+        <v>324000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <f>Raw_Sales_Data!H12*Raw_Sales_Data!G12</f>
+        <v>96000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <f>Raw_Sales_Data!H13*Raw_Sales_Data!G13</f>
+        <v>95000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <f>Raw_Sales_Data!H14*Raw_Sales_Data!G14</f>
+        <v>92000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <f>Raw_Sales_Data!H15*Raw_Sales_Data!G15</f>
+        <v>33600</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <f>Raw_Sales_Data!H16*Raw_Sales_Data!G16</f>
+        <v>165000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <f>Raw_Sales_Data!H17*Raw_Sales_Data!G17</f>
+        <v>125000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <f>Raw_Sales_Data!H18*Raw_Sales_Data!G18</f>
+        <v>38400</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <f>Raw_Sales_Data!H19*Raw_Sales_Data!G19</f>
+        <v>52500</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <f>Raw_Sales_Data!H20*Raw_Sales_Data!G20</f>
+        <v>54000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <f>Raw_Sales_Data!H21*Raw_Sales_Data!G21</f>
+        <v>36000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <f>Raw_Sales_Data!H22*Raw_Sales_Data!G22</f>
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <f>Raw_Sales_Data!H23*Raw_Sales_Data!G23</f>
+        <v>115000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <f>Raw_Sales_Data!H24*Raw_Sales_Data!G24</f>
+        <v>176000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <f>Raw_Sales_Data!H25*Raw_Sales_Data!G25</f>
+        <v>46800</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <f>Raw_Sales_Data!H26*Raw_Sales_Data!G26</f>
+        <v>136000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <f>Raw_Sales_Data!H27*Raw_Sales_Data!G27</f>
+        <v>63000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <f>Raw_Sales_Data!H28*Raw_Sales_Data!G28</f>
+        <v>49200</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <f>Raw_Sales_Data!H29*Raw_Sales_Data!G29</f>
+        <v>126000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <f>Raw_Sales_Data!H30*Raw_Sales_Data!G30</f>
+        <v>208000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <f>Raw_Sales_Data!H31*Raw_Sales_Data!G31</f>
+        <v>54400</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <f>Raw_Sales_Data!H32*Raw_Sales_Data!G32</f>
+        <v>230000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <f>Raw_Sales_Data!H33*Raw_Sales_Data!G33</f>
+        <v>135000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <f>Raw_Sales_Data!H34*Raw_Sales_Data!G34</f>
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <f>Raw_Sales_Data!H35*Raw_Sales_Data!G35</f>
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <f>Raw_Sales_Data!H36*Raw_Sales_Data!G36</f>
+        <v>184000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <f>Raw_Sales_Data!H37*Raw_Sales_Data!G37</f>
+        <v>86400</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <f>Raw_Sales_Data!H38*Raw_Sales_Data!G38</f>
+        <v>61600</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <f>Raw_Sales_Data!H39*Raw_Sales_Data!G39</f>
+        <v>108000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <f>Raw_Sales_Data!H40*Raw_Sales_Data!G40</f>
+        <v>270000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <f>Raw_Sales_Data!H41*Raw_Sales_Data!G41</f>
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <f>Raw_Sales_Data!H42*Raw_Sales_Data!G42</f>
+        <v>177000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <f>Raw_Sales_Data!H43*Raw_Sales_Data!G43</f>
+        <v>126000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <f>Raw_Sales_Data!H44*Raw_Sales_Data!G44</f>
+        <v>58300</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <f>Raw_Sales_Data!H45*Raw_Sales_Data!G45</f>
+        <v>195000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <f>Raw_Sales_Data!H46*Raw_Sales_Data!G46</f>
+        <v>324000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <f>Raw_Sales_Data!H47*Raw_Sales_Data!G47</f>
+        <v>43000</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <f>Raw_Sales_Data!H48*Raw_Sales_Data!G48</f>
+        <v>172000</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <f>Raw_Sales_Data!H49*Raw_Sales_Data!G49</f>
+        <v>141000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <f>Raw_Sales_Data!H50*Raw_Sales_Data!G50</f>
+        <v>89600</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <f>Raw_Sales_Data!H51*Raw_Sales_Data!G51</f>
+        <v>256000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
04 Completed Excel Questions 6-8
</commit_message>
<xml_diff>
--- a/sales-dataset.xlsx
+++ b/sales-dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\franc\OneDrive\Desktop\DATA SCIENCE\20 Beginner Excel Data Analyst Practice Questions\20_beginner_excel_data_analyst_practice_questions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B870353A-4F69-4440-A95A-24B5EC5931CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C39A1E6F-563D-49AD-960A-09E4441C7769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="102">
   <si>
     <t>Order_ID</t>
   </si>
@@ -334,6 +334,18 @@
   </si>
   <si>
     <t>Highest_Order_Value</t>
+  </si>
+  <si>
+    <t>Lowest_Order_Value</t>
+  </si>
+  <si>
+    <t>Count_Non_Empty_Total Orders</t>
+  </si>
+  <si>
+    <t>Count_Total_Orders</t>
+  </si>
+  <si>
+    <t>Count_Orders_By_City</t>
   </si>
 </sst>
 </file>
@@ -2378,11 +2390,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{754E7F86-FEF9-4E04-B3AF-20B05D640C6F}">
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="22.33203125" customWidth="1"/>
+    <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2490,12 +2502,19 @@
         <f>Raw_Sales_Data!H13*Raw_Sales_Data!G13</f>
         <v>95000</v>
       </c>
+      <c r="B13" s="4" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14">
         <f>Raw_Sales_Data!H14*Raw_Sales_Data!G14</f>
         <v>92000</v>
       </c>
+      <c r="B14">
+        <f>MIN(A2:A51)</f>
+        <v>25000</v>
+      </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15">
@@ -2508,98 +2527,139 @@
         <f>Raw_Sales_Data!H16*Raw_Sales_Data!G16</f>
         <v>165000</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B16" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <f>Raw_Sales_Data!H17*Raw_Sales_Data!G17</f>
         <v>125000</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B17">
+        <f>COUNT(A2:A51)</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <f>Raw_Sales_Data!H18*Raw_Sales_Data!G18</f>
         <v>38400</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <f>Raw_Sales_Data!H19*Raw_Sales_Data!G19</f>
         <v>52500</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B19" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20">
         <f>Raw_Sales_Data!H20*Raw_Sales_Data!G20</f>
         <v>54000</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B20">
+        <f>COUNTA(A2:A51)</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21">
         <f>Raw_Sales_Data!H21*Raw_Sales_Data!G21</f>
         <v>36000</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
         <f>Raw_Sales_Data!H22*Raw_Sales_Data!G22</f>
         <v>90000</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B22" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <f>Raw_Sales_Data!H23*Raw_Sales_Data!G23</f>
         <v>115000</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B23">
+        <f>COUNTIF(Raw_Sales_Data!D:D,Analysis!C23)</f>
+        <v>20</v>
+      </c>
+      <c r="C23" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
         <f>Raw_Sales_Data!H24*Raw_Sales_Data!G24</f>
         <v>176000</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B24">
+        <f>COUNTIF(Raw_Sales_Data!D:D,Analysis!C24)</f>
+        <v>17</v>
+      </c>
+      <c r="C24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <f>Raw_Sales_Data!H25*Raw_Sales_Data!G25</f>
         <v>46800</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B25">
+        <f>COUNTIF(Raw_Sales_Data!D:D,Analysis!C25)</f>
+        <v>13</v>
+      </c>
+      <c r="C25" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
         <f>Raw_Sales_Data!H26*Raw_Sales_Data!G26</f>
         <v>136000</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
         <f>Raw_Sales_Data!H27*Raw_Sales_Data!G27</f>
         <v>63000</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28">
         <f>Raw_Sales_Data!H28*Raw_Sales_Data!G28</f>
         <v>49200</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <f>Raw_Sales_Data!H29*Raw_Sales_Data!G29</f>
         <v>126000</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
         <f>Raw_Sales_Data!H30*Raw_Sales_Data!G30</f>
         <v>208000</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <f>Raw_Sales_Data!H31*Raw_Sales_Data!G31</f>
         <v>54400</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <f>Raw_Sales_Data!H32*Raw_Sales_Data!G32</f>
         <v>230000</v>

</xml_diff>